<commit_message>
Robô de Comissões com a lógica de recebimentos por adiantamentos ou recebimentos normais implementada!
</commit_message>
<xml_diff>
--- a/Analise_Comercial_Completa.xlsx
+++ b/Analise_Comercial_Completa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m.rafael\Desktop\projetos\robo-comissoes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6523894-84D4-4EDB-8A17-0C6EAF9846F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{447F0727-AAE0-45FE-86CD-FDC807156E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="32">
   <si>
     <t>Processo</t>
   </si>
@@ -114,10 +114,13 @@
     <t>Base Teste FC</t>
   </si>
   <si>
-    <t>Cliente Teste</t>
-  </si>
-  <si>
-    <t>FC-Base3</t>
+    <t>005309</t>
+  </si>
+  <si>
+    <t>Numero NF</t>
+  </si>
+  <si>
+    <t>048341</t>
   </si>
 </sst>
 </file>
@@ -446,15 +449,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="32.85546875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -509,10 +513,13 @@
       <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="S1" s="1" t="s">
+        <v>30</v>
+      </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>30</v>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>999999</v>
       </c>
       <c r="B2" s="2">
         <v>45915</v>
@@ -559,8 +566,67 @@
       <c r="P2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="R2" s="1" t="s">
+      <c r="R2" t="s">
         <v>29</v>
+      </c>
+      <c r="S2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>999998</v>
+      </c>
+      <c r="B3" s="2">
+        <v>45915</v>
+      </c>
+      <c r="C3" s="2">
+        <v>45915</v>
+      </c>
+      <c r="D3" s="1">
+        <v>100</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="L3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="O3" s="1">
+        <v>0</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R3" t="s">
+        <v>29</v>
+      </c>
+      <c r="S3" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FRONTEND 1.0 PRATICAMENTE PRONTO - COM INTERFACE PARA CROSS-SELLING
</commit_message>
<xml_diff>
--- a/Analise_Comercial_Completa.xlsx
+++ b/Analise_Comercial_Completa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m.rafael\Desktop\projetos\robo-comissoes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{447F0727-AAE0-45FE-86CD-FDC807156E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6DB8C68-8AFB-4BA6-83B7-61F3471E1C48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="40">
   <si>
     <t>Processo</t>
   </si>
@@ -121,6 +121,30 @@
   </si>
   <si>
     <t>048341</t>
+  </si>
+  <si>
+    <t>CS-Test</t>
+  </si>
+  <si>
+    <t>Sensor</t>
+  </si>
+  <si>
+    <t>Reposição</t>
+  </si>
+  <si>
+    <t>ROSILENE</t>
+  </si>
+  <si>
+    <t>HON-SENS-CS</t>
+  </si>
+  <si>
+    <t>Teste Cross Selling</t>
+  </si>
+  <si>
+    <t>MATEUS BORRO MACHADO</t>
+  </si>
+  <si>
+    <t>Cliente CS</t>
   </si>
 </sst>
 </file>
@@ -449,11 +473,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="32.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
@@ -629,6 +654,62 @@
         <v>31</v>
       </c>
     </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="2">
+        <v>45920</v>
+      </c>
+      <c r="C4" s="2">
+        <v>45920</v>
+      </c>
+      <c r="D4" s="1">
+        <v>100</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L4" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="O4" s="1">
+        <v>100</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>38</v>
+      </c>
+      <c r="R4" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>